<commit_message>
Improve consent auth and chat recording UX
</commit_message>
<xml_diff>
--- a/data/ndhu-learning-warning-schema.xlsx
+++ b/data/ndhu-learning-warning-schema.xlsx
@@ -2,18 +2,18 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="1" r:id="R8c307d778fd94e65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CollegesDepartments" sheetId="2" r:id="R5a36c1f16a914d02"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="3" r:id="R5b6da3812dc84c43"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teachers" sheetId="4" r:id="R024a2884a576445c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LearningCheckins" sheetId="5" r:id="Redafc87f25634482"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conversations" sheetId="6" r:id="Ra81dacf2feed4e98"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RiskSignals" sheetId="7" r:id="R9221d6d0b8f34426"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InterventionPlans" sheetId="8" r:id="Rfe60715c31c24795"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TeacherNotes" sheetId="9" r:id="R3c4fde2e3c10448d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referrals" sheetId="10" r:id="Rc59fbcda36504126"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="11" r:id="R92ae1a3206d2400b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AnalyticsDashboard" sheetId="12" r:id="R38c7ce9bc70e49ad"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Settings" sheetId="1" r:id="Re870abd4bc894b87"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CollegesDepartments" sheetId="2" r:id="R249b966767794f96"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Students" sheetId="3" r:id="R530641bc981044d9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Teachers" sheetId="4" r:id="R05c1ba75941b4c0a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="LearningCheckins" sheetId="5" r:id="R286e50aea6be4f61"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Conversations" sheetId="6" r:id="R2c28315d12f94874"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="RiskSignals" sheetId="7" r:id="Rcef376d4eb694297"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="InterventionPlans" sheetId="8" r:id="Racf815b6834a41bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="TeacherNotes" sheetId="9" r:id="Rfc1616379a904ba5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Referrals" sheetId="10" r:id="R8f13ece286fa4447"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AuditLog" sheetId="11" r:id="Rf117775eb08b415e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="AnalyticsDashboard" sheetId="12" r:id="Reb0d43954d6146bc"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -249,13 +249,13 @@
         <x:v>app_name</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>東華大學學生學習預警輔導系統</x:v>
+        <x:v>國立東華大學學習關懷預警系統</x:v>
       </x:c>
       <x:c r="C2" t="str">
         <x:v>系統名稱</x:v>
       </x:c>
       <x:c r="D2" t="n">
-        <x:v>46146.0530255787</x:v>
+        <x:v>46146.25445263889</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="21" customHeight="1">
@@ -269,7 +269,7 @@
         <x:v>教師端與學生端共同使用的關懷層級</x:v>
       </x:c>
       <x:c r="D3" t="n">
-        <x:v>46146.0530255787</x:v>
+        <x:v>46146.25445263889</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="21" customHeight="1">
@@ -281,7 +281,7 @@
         <x:v>部署 Apps Script 後填入</x:v>
       </x:c>
       <x:c r="D4" t="n">
-        <x:v>46146.0530255787</x:v>
+        <x:v>46146.25445263889</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="21" customHeight="1">
@@ -295,7 +295,7 @@
         <x:v>若 GAS 設定 OPENAI_API_KEY，可用於風險摘要與建議</x:v>
       </x:c>
       <x:c r="D5" t="n">
-        <x:v>46146.0530255787</x:v>
+        <x:v>46146.25445263889</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="21" customHeight="1">
@@ -309,7 +309,7 @@
         <x:v>教師端預設只看摘要，不直接顯示完整對話</x:v>
       </x:c>
       <x:c r="D6" t="n">
-        <x:v>46146.0530255787</x:v>
+        <x:v>46146.25445263889</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -443,7 +443,7 @@
         <x:v>Students!A2:A5000</x:v>
       </x:c>
       <x:c r="D2" t="n">
-        <x:v>46146.05302703704</x:v>
+        <x:v>46146.25445501157</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="21" customHeight="1">
@@ -458,7 +458,7 @@
         <x:v>Students!L2:L5000</x:v>
       </x:c>
       <x:c r="D3" t="n">
-        <x:v>46146.05302703704</x:v>
+        <x:v>46146.25445501157</x:v>
       </x:c>
     </x:row>
     <x:row r="4" ht="21" customHeight="1">
@@ -473,7 +473,7 @@
         <x:v>Students!L2:L5000</x:v>
       </x:c>
       <x:c r="D4" t="n">
-        <x:v>46146.05302703704</x:v>
+        <x:v>46146.25445501157</x:v>
       </x:c>
     </x:row>
     <x:row r="5" ht="21" customHeight="1">
@@ -488,7 +488,7 @@
         <x:v>Students!L2:L5000</x:v>
       </x:c>
       <x:c r="D5" t="n">
-        <x:v>46146.05302703704</x:v>
+        <x:v>46146.25445501157</x:v>
       </x:c>
     </x:row>
     <x:row r="6" ht="21" customHeight="1">
@@ -503,7 +503,7 @@
         <x:v>LearningCheckins!A2:A5000</x:v>
       </x:c>
       <x:c r="D6" t="n">
-        <x:v>46146.05302703704</x:v>
+        <x:v>46146.25445501157</x:v>
       </x:c>
     </x:row>
     <x:row r="7" ht="21" customHeight="1">
@@ -518,7 +518,7 @@
         <x:v>TeacherNotes!A2:A5000</x:v>
       </x:c>
       <x:c r="D7" t="n">
-        <x:v>46146.05302703704</x:v>
+        <x:v>46146.25445501157</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -559,13 +559,13 @@
         <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>中國語文學系</x:v>
+        <x:v>諮商與臨床心理學系</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>學士/碩士/博士</x:v>
+        <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E2" t="str">
         <x:v>TRUE</x:v>
@@ -582,7 +582,7 @@
         <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E3" t="str">
         <x:v>TRUE</x:v>
@@ -593,13 +593,13 @@
         <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>英美語文學系</x:v>
+        <x:v>中國語文學系</x:v>
       </x:c>
       <x:c r="C4" t="str">
         <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E4" t="str">
         <x:v>TRUE</x:v>
@@ -610,13 +610,13 @@
         <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>臺灣文化學系</x:v>
+        <x:v>英美語文學系</x:v>
       </x:c>
       <x:c r="C5" t="str">
         <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E5" t="str">
         <x:v>TRUE</x:v>
@@ -627,13 +627,13 @@
         <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>歷史學系</x:v>
+        <x:v>臺灣文化學系</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E6" t="str">
         <x:v>TRUE</x:v>
@@ -644,13 +644,13 @@
         <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>社會學系</x:v>
+        <x:v>歷史學系</x:v>
       </x:c>
       <x:c r="C7" t="str">
         <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E7" t="str">
         <x:v>TRUE</x:v>
@@ -661,13 +661,13 @@
         <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B8" t="str">
-        <x:v>公共行政學系</x:v>
+        <x:v>經濟學系</x:v>
       </x:c>
       <x:c r="C8" t="str">
         <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D8" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E8" t="str">
         <x:v>TRUE</x:v>
@@ -678,13 +678,13 @@
         <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B9" t="str">
-        <x:v>經濟學系</x:v>
+        <x:v>社會學系</x:v>
       </x:c>
       <x:c r="C9" t="str">
         <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D9" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E9" t="str">
         <x:v>TRUE</x:v>
@@ -695,13 +695,13 @@
         <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B10" t="str">
-        <x:v>法律學系</x:v>
+        <x:v>公共行政學系</x:v>
       </x:c>
       <x:c r="C10" t="str">
-        <x:v>學士</x:v>
+        <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D10" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E10" t="str">
         <x:v>TRUE</x:v>
@@ -709,16 +709,16 @@
     </x:row>
     <x:row r="11" ht="21" customHeight="1">
       <x:c r="A11" t="str">
-        <x:v>理工學院</x:v>
+        <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B11" t="str">
-        <x:v>應用數學系</x:v>
+        <x:v>法律學系（含原住民專班）</x:v>
       </x:c>
       <x:c r="C11" t="str">
-        <x:v>學士/碩士/博士</x:v>
+        <x:v>學士</x:v>
       </x:c>
       <x:c r="D11" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E11" t="str">
         <x:v>TRUE</x:v>
@@ -726,16 +726,16 @@
     </x:row>
     <x:row r="12" ht="21" customHeight="1">
       <x:c r="A12" t="str">
-        <x:v>理工學院</x:v>
+        <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B12" t="str">
-        <x:v>物理學系</x:v>
+        <x:v>華語文教學國際博士班</x:v>
       </x:c>
       <x:c r="C12" t="str">
-        <x:v>學士/碩士/博士</x:v>
+        <x:v>博士</x:v>
       </x:c>
       <x:c r="D12" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E12" t="str">
         <x:v>TRUE</x:v>
@@ -743,16 +743,16 @@
     </x:row>
     <x:row r="13" ht="21" customHeight="1">
       <x:c r="A13" t="str">
-        <x:v>理工學院</x:v>
+        <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B13" t="str">
-        <x:v>化學系</x:v>
+        <x:v>亞太區域研究博士班</x:v>
       </x:c>
       <x:c r="C13" t="str">
-        <x:v>學士/碩士/博士</x:v>
+        <x:v>博士</x:v>
       </x:c>
       <x:c r="D13" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E13" t="str">
         <x:v>TRUE</x:v>
@@ -760,16 +760,16 @@
     </x:row>
     <x:row r="14" ht="21" customHeight="1">
       <x:c r="A14" t="str">
-        <x:v>理工學院</x:v>
+        <x:v>人文社會科學學院</x:v>
       </x:c>
       <x:c r="B14" t="str">
-        <x:v>生命科學系</x:v>
+        <x:v>華語文教學暨書法國際碩士班</x:v>
       </x:c>
       <x:c r="C14" t="str">
-        <x:v>學士/碩士/博士</x:v>
+        <x:v>碩士</x:v>
       </x:c>
       <x:c r="D14" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E14" t="str">
         <x:v>TRUE</x:v>
@@ -780,13 +780,13 @@
         <x:v>理工學院</x:v>
       </x:c>
       <x:c r="B15" t="str">
-        <x:v>電機工程學系</x:v>
+        <x:v>應用數學系</x:v>
       </x:c>
       <x:c r="C15" t="str">
         <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D15" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E15" t="str">
         <x:v>TRUE</x:v>
@@ -797,13 +797,13 @@
         <x:v>理工學院</x:v>
       </x:c>
       <x:c r="B16" t="str">
-        <x:v>資訊工程學系</x:v>
+        <x:v>物理學系</x:v>
       </x:c>
       <x:c r="C16" t="str">
         <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D16" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E16" t="str">
         <x:v>TRUE</x:v>
@@ -814,13 +814,13 @@
         <x:v>理工學院</x:v>
       </x:c>
       <x:c r="B17" t="str">
-        <x:v>材料科學與工程學系</x:v>
+        <x:v>生化暨分子醫學科學系</x:v>
       </x:c>
       <x:c r="C17" t="str">
         <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D17" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E17" t="str">
         <x:v>TRUE</x:v>
@@ -831,13 +831,13 @@
         <x:v>理工學院</x:v>
       </x:c>
       <x:c r="B18" t="str">
-        <x:v>光電工程學系</x:v>
+        <x:v>化學系</x:v>
       </x:c>
       <x:c r="C18" t="str">
         <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D18" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E18" t="str">
         <x:v>TRUE</x:v>
@@ -845,16 +845,16 @@
     </x:row>
     <x:row r="19" ht="21" customHeight="1">
       <x:c r="A19" t="str">
-        <x:v>管理學院</x:v>
+        <x:v>理工學院</x:v>
       </x:c>
       <x:c r="B19" t="str">
-        <x:v>企業管理學系</x:v>
+        <x:v>光電工程學系</x:v>
       </x:c>
       <x:c r="C19" t="str">
         <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D19" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E19" t="str">
         <x:v>TRUE</x:v>
@@ -862,16 +862,16 @@
     </x:row>
     <x:row r="20" ht="21" customHeight="1">
       <x:c r="A20" t="str">
-        <x:v>管理學院</x:v>
+        <x:v>理工學院</x:v>
       </x:c>
       <x:c r="B20" t="str">
-        <x:v>國際企業學系</x:v>
+        <x:v>電機工程學系</x:v>
       </x:c>
       <x:c r="C20" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D20" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E20" t="str">
         <x:v>TRUE</x:v>
@@ -879,16 +879,16 @@
     </x:row>
     <x:row r="21" ht="21" customHeight="1">
       <x:c r="A21" t="str">
-        <x:v>管理學院</x:v>
+        <x:v>理工學院</x:v>
       </x:c>
       <x:c r="B21" t="str">
-        <x:v>會計學系</x:v>
+        <x:v>資訊工程學系</x:v>
       </x:c>
       <x:c r="C21" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D21" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E21" t="str">
         <x:v>TRUE</x:v>
@@ -896,16 +896,16 @@
     </x:row>
     <x:row r="22" ht="21" customHeight="1">
       <x:c r="A22" t="str">
-        <x:v>管理學院</x:v>
+        <x:v>理工學院</x:v>
       </x:c>
       <x:c r="B22" t="str">
-        <x:v>財務金融學系</x:v>
+        <x:v>材料科學與工程學系</x:v>
       </x:c>
       <x:c r="C22" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D22" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E22" t="str">
         <x:v>TRUE</x:v>
@@ -913,16 +913,16 @@
     </x:row>
     <x:row r="23" ht="21" customHeight="1">
       <x:c r="A23" t="str">
-        <x:v>管理學院</x:v>
+        <x:v>理工學院</x:v>
       </x:c>
       <x:c r="B23" t="str">
-        <x:v>資訊管理學系</x:v>
+        <x:v>大數據科學國際學士班</x:v>
       </x:c>
       <x:c r="C23" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士</x:v>
       </x:c>
       <x:c r="D23" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E23" t="str">
         <x:v>TRUE</x:v>
@@ -933,13 +933,13 @@
         <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B24" t="str">
-        <x:v>觀光暨休閒遊憩學系</x:v>
+        <x:v>企業管理學系</x:v>
       </x:c>
       <x:c r="C24" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D24" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E24" t="str">
         <x:v>TRUE</x:v>
@@ -950,13 +950,13 @@
         <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B25" t="str">
-        <x:v>管理科學與財金國際學士學位學程</x:v>
+        <x:v>運籌管理研究所</x:v>
       </x:c>
       <x:c r="C25" t="str">
-        <x:v>學士</x:v>
+        <x:v>碩士/博士</x:v>
       </x:c>
       <x:c r="D25" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E25" t="str">
         <x:v>TRUE</x:v>
@@ -964,16 +964,16 @@
     </x:row>
     <x:row r="26" ht="21" customHeight="1">
       <x:c r="A26" t="str">
-        <x:v>花師教育學院</x:v>
+        <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B26" t="str">
-        <x:v>教育與潛能開發學系</x:v>
+        <x:v>國際企業學系</x:v>
       </x:c>
       <x:c r="C26" t="str">
-        <x:v>學士/碩士/博士</x:v>
+        <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D26" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E26" t="str">
         <x:v>TRUE</x:v>
@@ -981,16 +981,16 @@
     </x:row>
     <x:row r="27" ht="21" customHeight="1">
       <x:c r="A27" t="str">
-        <x:v>花師教育學院</x:v>
+        <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B27" t="str">
-        <x:v>教育行政與管理學系</x:v>
+        <x:v>會計學系</x:v>
       </x:c>
       <x:c r="C27" t="str">
-        <x:v>學士/碩士/博士</x:v>
+        <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D27" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E27" t="str">
         <x:v>TRUE</x:v>
@@ -998,16 +998,16 @@
     </x:row>
     <x:row r="28" ht="21" customHeight="1">
       <x:c r="A28" t="str">
-        <x:v>花師教育學院</x:v>
+        <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B28" t="str">
-        <x:v>特殊教育學系</x:v>
+        <x:v>資訊管理學系</x:v>
       </x:c>
       <x:c r="C28" t="str">
-        <x:v>學士/碩士/博士</x:v>
+        <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D28" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E28" t="str">
         <x:v>TRUE</x:v>
@@ -1015,16 +1015,16 @@
     </x:row>
     <x:row r="29" ht="21" customHeight="1">
       <x:c r="A29" t="str">
-        <x:v>花師教育學院</x:v>
+        <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B29" t="str">
-        <x:v>幼兒教育學系</x:v>
+        <x:v>財務金融學系</x:v>
       </x:c>
       <x:c r="C29" t="str">
         <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D29" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E29" t="str">
         <x:v>TRUE</x:v>
@@ -1032,16 +1032,16 @@
     </x:row>
     <x:row r="30" ht="21" customHeight="1">
       <x:c r="A30" t="str">
-        <x:v>花師教育學院</x:v>
+        <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B30" t="str">
-        <x:v>體育與運動科學系</x:v>
+        <x:v>觀光暨休閒遊憩學系</x:v>
       </x:c>
       <x:c r="C30" t="str">
         <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D30" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E30" t="str">
         <x:v>TRUE</x:v>
@@ -1049,16 +1049,16 @@
     </x:row>
     <x:row r="31" ht="21" customHeight="1">
       <x:c r="A31" t="str">
-        <x:v>花師教育學院</x:v>
+        <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B31" t="str">
-        <x:v>諮商與臨床心理學系</x:v>
+        <x:v>高階經營管理碩士在職專班</x:v>
       </x:c>
       <x:c r="C31" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>碩士</x:v>
       </x:c>
       <x:c r="D31" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E31" t="str">
         <x:v>TRUE</x:v>
@@ -1066,16 +1066,16 @@
     </x:row>
     <x:row r="32" ht="21" customHeight="1">
       <x:c r="A32" t="str">
-        <x:v>藝術學院</x:v>
+        <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B32" t="str">
-        <x:v>音樂學系</x:v>
+        <x:v>管理科學與財金國際學士學位學程</x:v>
       </x:c>
       <x:c r="C32" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士</x:v>
       </x:c>
       <x:c r="D32" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E32" t="str">
         <x:v>TRUE</x:v>
@@ -1083,16 +1083,16 @@
     </x:row>
     <x:row r="33" ht="21" customHeight="1">
       <x:c r="A33" t="str">
-        <x:v>藝術學院</x:v>
+        <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B33" t="str">
-        <x:v>藝術與設計學系</x:v>
+        <x:v>會計與資訊管理國際學士班</x:v>
       </x:c>
       <x:c r="C33" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士</x:v>
       </x:c>
       <x:c r="D33" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E33" t="str">
         <x:v>TRUE</x:v>
@@ -1100,16 +1100,16 @@
     </x:row>
     <x:row r="34" ht="21" customHeight="1">
       <x:c r="A34" t="str">
-        <x:v>藝術學院</x:v>
+        <x:v>管理學院</x:v>
       </x:c>
       <x:c r="B34" t="str">
-        <x:v>藝術創意產業學系</x:v>
+        <x:v>數位行銷與服務創新國際學士班</x:v>
       </x:c>
       <x:c r="C34" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士</x:v>
       </x:c>
       <x:c r="D34" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E34" t="str">
         <x:v>TRUE</x:v>
@@ -1117,16 +1117,16 @@
     </x:row>
     <x:row r="35" ht="21" customHeight="1">
       <x:c r="A35" t="str">
-        <x:v>原住民民族學院</x:v>
+        <x:v>花師教育學院</x:v>
       </x:c>
       <x:c r="B35" t="str">
-        <x:v>民族語言與傳播學系</x:v>
+        <x:v>教育與潛能開發學系</x:v>
       </x:c>
       <x:c r="C35" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D35" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E35" t="str">
         <x:v>TRUE</x:v>
@@ -1134,16 +1134,16 @@
     </x:row>
     <x:row r="36" ht="21" customHeight="1">
       <x:c r="A36" t="str">
-        <x:v>原住民民族學院</x:v>
+        <x:v>花師教育學院</x:v>
       </x:c>
       <x:c r="B36" t="str">
-        <x:v>民族事務與發展學系</x:v>
+        <x:v>教育行政與管理學系</x:v>
       </x:c>
       <x:c r="C36" t="str">
-        <x:v>學士/碩士</x:v>
+        <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D36" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E36" t="str">
         <x:v>TRUE</x:v>
@@ -1151,16 +1151,16 @@
     </x:row>
     <x:row r="37" ht="21" customHeight="1">
       <x:c r="A37" t="str">
-        <x:v>原住民民族學院</x:v>
+        <x:v>花師教育學院</x:v>
       </x:c>
       <x:c r="B37" t="str">
-        <x:v>民族社會工作學士學位學程</x:v>
+        <x:v>特殊教育學系</x:v>
       </x:c>
       <x:c r="C37" t="str">
-        <x:v>學士</x:v>
+        <x:v>學士/碩士/博士</x:v>
       </x:c>
       <x:c r="D37" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E37" t="str">
         <x:v>TRUE</x:v>
@@ -1168,16 +1168,16 @@
     </x:row>
     <x:row r="38" ht="21" customHeight="1">
       <x:c r="A38" t="str">
-        <x:v>原住民民族學院</x:v>
+        <x:v>花師教育學院</x:v>
       </x:c>
       <x:c r="B38" t="str">
-        <x:v>原住民族樂舞與藝術學士學位學程</x:v>
+        <x:v>體育與運動科學系</x:v>
       </x:c>
       <x:c r="C38" t="str">
-        <x:v>學士</x:v>
+        <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D38" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E38" t="str">
         <x:v>TRUE</x:v>
@@ -1185,16 +1185,16 @@
     </x:row>
     <x:row r="39" ht="21" customHeight="1">
       <x:c r="A39" t="str">
-        <x:v>環境暨海洋學院</x:v>
+        <x:v>花師教育學院</x:v>
       </x:c>
       <x:c r="B39" t="str">
-        <x:v>自然資源與環境學系</x:v>
+        <x:v>幼兒教育學系</x:v>
       </x:c>
       <x:c r="C39" t="str">
-        <x:v>學士/碩士/博士</x:v>
+        <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D39" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E39" t="str">
         <x:v>TRUE</x:v>
@@ -1202,16 +1202,16 @@
     </x:row>
     <x:row r="40" ht="21" customHeight="1">
       <x:c r="A40" t="str">
-        <x:v>環境暨海洋學院</x:v>
+        <x:v>花師教育學院</x:v>
       </x:c>
       <x:c r="B40" t="str">
-        <x:v>海洋生物研究所</x:v>
+        <x:v>多元文化教育碩博士班</x:v>
       </x:c>
       <x:c r="C40" t="str">
         <x:v>碩士/博士</x:v>
       </x:c>
       <x:c r="D40" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E40" t="str">
         <x:v>TRUE</x:v>
@@ -1219,16 +1219,16 @@
     </x:row>
     <x:row r="41" ht="21" customHeight="1">
       <x:c r="A41" t="str">
-        <x:v>洄瀾學院</x:v>
+        <x:v>藝術學院</x:v>
       </x:c>
       <x:c r="B41" t="str">
-        <x:v>縱谷跨域書院學士學位學程</x:v>
+        <x:v>音樂學系</x:v>
       </x:c>
       <x:c r="C41" t="str">
-        <x:v>學士</x:v>
+        <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D41" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E41" t="str">
         <x:v>TRUE</x:v>
@@ -1236,16 +1236,16 @@
     </x:row>
     <x:row r="42" ht="21" customHeight="1">
       <x:c r="A42" t="str">
-        <x:v>洄瀾學院</x:v>
+        <x:v>藝術學院</x:v>
       </x:c>
       <x:c r="B42" t="str">
-        <x:v>人文與科學跨領域學士學位學程</x:v>
+        <x:v>藝術與設計學系</x:v>
       </x:c>
       <x:c r="C42" t="str">
-        <x:v>學士</x:v>
+        <x:v>學士/碩士</x:v>
       </x:c>
       <x:c r="D42" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
       </x:c>
       <x:c r="E42" t="str">
         <x:v>TRUE</x:v>
@@ -1253,18 +1253,290 @@
     </x:row>
     <x:row r="43" ht="21" customHeight="1">
       <x:c r="A43" t="str">
+        <x:v>藝術學院</x:v>
+      </x:c>
+      <x:c r="B43" t="str">
+        <x:v>藝術創意產業學系</x:v>
+      </x:c>
+      <x:c r="C43" t="str">
+        <x:v>學士/碩士</x:v>
+      </x:c>
+      <x:c r="D43" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E43" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="44" ht="21" customHeight="1">
+      <x:c r="A44" t="str">
+        <x:v>藝術學院</x:v>
+      </x:c>
+      <x:c r="B44" t="str">
+        <x:v>藝術跨領域國際博士班</x:v>
+      </x:c>
+      <x:c r="C44" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D44" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E44" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="45" ht="21" customHeight="1">
+      <x:c r="A45" t="str">
+        <x:v>原住民民族學院</x:v>
+      </x:c>
+      <x:c r="B45" t="str">
+        <x:v>族群關係與文化學系</x:v>
+      </x:c>
+      <x:c r="C45" t="str">
+        <x:v>學士/碩士</x:v>
+      </x:c>
+      <x:c r="D45" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E45" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="46" ht="21" customHeight="1">
+      <x:c r="A46" t="str">
+        <x:v>原住民民族學院</x:v>
+      </x:c>
+      <x:c r="B46" t="str">
+        <x:v>民族語言與傳播學系</x:v>
+      </x:c>
+      <x:c r="C46" t="str">
+        <x:v>學士/碩士</x:v>
+      </x:c>
+      <x:c r="D46" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E46" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="47" ht="21" customHeight="1">
+      <x:c r="A47" t="str">
+        <x:v>原住民民族學院</x:v>
+      </x:c>
+      <x:c r="B47" t="str">
+        <x:v>民族發展與社會工作學系</x:v>
+      </x:c>
+      <x:c r="C47" t="str">
+        <x:v>學士/碩士</x:v>
+      </x:c>
+      <x:c r="D47" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E47" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="48" ht="21" customHeight="1">
+      <x:c r="A48" t="str">
+        <x:v>原住民民族學院</x:v>
+      </x:c>
+      <x:c r="B48" t="str">
+        <x:v>民族社會工作學士學位學程</x:v>
+      </x:c>
+      <x:c r="C48" t="str">
+        <x:v>學士</x:v>
+      </x:c>
+      <x:c r="D48" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E48" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="49" ht="21" customHeight="1">
+      <x:c r="A49" t="str">
+        <x:v>原住民民族學院</x:v>
+      </x:c>
+      <x:c r="B49" t="str">
+        <x:v>原住民族樂舞與藝術學士學位學程</x:v>
+      </x:c>
+      <x:c r="C49" t="str">
+        <x:v>學士</x:v>
+      </x:c>
+      <x:c r="D49" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E49" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="50" ht="21" customHeight="1">
+      <x:c r="A50" t="str">
+        <x:v>原住民民族學院</x:v>
+      </x:c>
+      <x:c r="B50" t="str">
+        <x:v>原住民族研究國際博士班</x:v>
+      </x:c>
+      <x:c r="C50" t="str">
+        <x:v>博士</x:v>
+      </x:c>
+      <x:c r="D50" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E50" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="51" ht="21" customHeight="1">
+      <x:c r="A51" t="str">
+        <x:v>環境暨海洋學院</x:v>
+      </x:c>
+      <x:c r="B51" t="str">
+        <x:v>自然資源與環境學系</x:v>
+      </x:c>
+      <x:c r="C51" t="str">
+        <x:v>學士/碩士/博士</x:v>
+      </x:c>
+      <x:c r="D51" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E51" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="52" ht="21" customHeight="1">
+      <x:c r="A52" t="str">
+        <x:v>環境暨海洋學院</x:v>
+      </x:c>
+      <x:c r="B52" t="str">
+        <x:v>海洋生物研究所</x:v>
+      </x:c>
+      <x:c r="C52" t="str">
+        <x:v>碩士/博士</x:v>
+      </x:c>
+      <x:c r="D52" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E52" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="53" ht="21" customHeight="1">
+      <x:c r="A53" t="str">
+        <x:v>環境暨海洋學院</x:v>
+      </x:c>
+      <x:c r="B53" t="str">
+        <x:v>人文與環境碩士學位學程</x:v>
+      </x:c>
+      <x:c r="C53" t="str">
+        <x:v>碩士</x:v>
+      </x:c>
+      <x:c r="D53" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E53" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="54" ht="21" customHeight="1">
+      <x:c r="A54" t="str">
         <x:v>洄瀾學院</x:v>
       </x:c>
-      <x:c r="B43" t="str">
+      <x:c r="B54" t="str">
         <x:v>通識教育中心</x:v>
       </x:c>
-      <x:c r="C43" t="str">
+      <x:c r="C54" t="str">
         <x:v>通識</x:v>
       </x:c>
-      <x:c r="D43" t="str">
-        <x:v>依東華招生與院系公開資訊整理，實際以教務處公告為準</x:v>
-      </x:c>
-      <x:c r="E43" t="str">
+      <x:c r="D54" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E54" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="55" ht="21" customHeight="1">
+      <x:c r="A55" t="str">
+        <x:v>洄瀾學院</x:v>
+      </x:c>
+      <x:c r="B55" t="str">
+        <x:v>藝文中心</x:v>
+      </x:c>
+      <x:c r="C55" t="str">
+        <x:v>中心</x:v>
+      </x:c>
+      <x:c r="D55" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E55" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="56" ht="21" customHeight="1">
+      <x:c r="A56" t="str">
+        <x:v>洄瀾學院</x:v>
+      </x:c>
+      <x:c r="B56" t="str">
+        <x:v>體育中心</x:v>
+      </x:c>
+      <x:c r="C56" t="str">
+        <x:v>中心</x:v>
+      </x:c>
+      <x:c r="D56" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E56" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="57" ht="21" customHeight="1">
+      <x:c r="A57" t="str">
+        <x:v>洄瀾學院</x:v>
+      </x:c>
+      <x:c r="B57" t="str">
+        <x:v>語言中心</x:v>
+      </x:c>
+      <x:c r="C57" t="str">
+        <x:v>中心</x:v>
+      </x:c>
+      <x:c r="D57" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E57" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="58" ht="21" customHeight="1">
+      <x:c r="A58" t="str">
+        <x:v>洄瀾學院</x:v>
+      </x:c>
+      <x:c r="B58" t="str">
+        <x:v>華語文中心</x:v>
+      </x:c>
+      <x:c r="C58" t="str">
+        <x:v>中心</x:v>
+      </x:c>
+      <x:c r="D58" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E58" t="str">
+        <x:v>TRUE</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="59" ht="21" customHeight="1">
+      <x:c r="A59" t="str">
+        <x:v>洄瀾學院</x:v>
+      </x:c>
+      <x:c r="B59" t="str">
+        <x:v>縱谷跨域書院學士學位學程</x:v>
+      </x:c>
+      <x:c r="C59" t="str">
+        <x:v>學士</x:v>
+      </x:c>
+      <x:c r="D59" t="str">
+        <x:v>依國立東華大學教學單位頁面整理，實際以校方公告為準</x:v>
+      </x:c>
+      <x:c r="E59" t="str">
         <x:v>TRUE</x:v>
       </x:c>
     </x:row>
@@ -1283,15 +1555,14 @@
     <x:col min="4" max="4" width="5.650000095367432" hidden="0" customWidth="1"/>
     <x:col min="5" max="5" width="9.6899995803833" hidden="0" customWidth="1"/>
     <x:col min="6" max="6" width="3.5" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="11.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="12.25" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="4.849999904632568" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="8.75" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="10.229999542236328" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="7.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="8.210000038146973" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="11.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="13.1899995803833" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="12.25" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="4.849999904632568" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8.75" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="10.229999542236328" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="7.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="8.210000038146973" hidden="0" customWidth="1"/>
+    <x:col min="13" max="13" width="11.4399995803833" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="13.1899995803833" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="21" customHeight="1">
@@ -1314,30 +1585,27 @@
         <x:v>year</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>advisor_email</x:v>
+        <x:v>consent_status</x:v>
       </x:c>
       <x:c r="H1" s="4" t="str">
-        <x:v>consent_status</x:v>
+        <x:v>status</x:v>
       </x:c>
       <x:c r="I1" s="4" t="str">
-        <x:v>status</x:v>
+        <x:v>created_at</x:v>
       </x:c>
       <x:c r="J1" s="4" t="str">
-        <x:v>created_at</x:v>
+        <x:v>last_seen_at</x:v>
       </x:c>
       <x:c r="K1" s="4" t="str">
-        <x:v>last_seen_at</x:v>
+        <x:v>risk_level</x:v>
       </x:c>
       <x:c r="L1" s="4" t="str">
-        <x:v>risk_level</x:v>
+        <x:v>risk_score</x:v>
       </x:c>
       <x:c r="M1" s="4" t="str">
-        <x:v>risk_score</x:v>
+        <x:v>primary_need</x:v>
       </x:c>
       <x:c r="N1" s="4" t="str">
-        <x:v>primary_need</x:v>
-      </x:c>
-      <x:c r="O1" s="4" t="str">
         <x:v>latest_summary</x:v>
       </x:c>
     </x:row>
@@ -1411,19 +1679,18 @@
     <x:col min="6" max="6" width="5.650000095367432" hidden="0" customWidth="1"/>
     <x:col min="7" max="7" width="9.6899995803833" hidden="0" customWidth="1"/>
     <x:col min="8" max="8" width="3.5" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="11.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="10.899999618530273" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="11.710000038146973" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="12.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="10.899999618530273" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="11.710000038146973" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="12.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="15.069999694824219" hidden="0" customWidth="1"/>
     <x:col min="13" max="13" width="15.069999694824219" hidden="0" customWidth="1"/>
-    <x:col min="14" max="14" width="15.069999694824219" hidden="0" customWidth="1"/>
-    <x:col min="15" max="15" width="12.789999961853027" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="7.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="17" max="17" width="8.210000038146973" hidden="0" customWidth="1"/>
-    <x:col min="18" max="18" width="3.2300000190734863" hidden="0" customWidth="1"/>
-    <x:col min="19" max="19" width="7.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="20" max="20" width="19.25" hidden="0" customWidth="1"/>
-    <x:col min="21" max="21" width="7.400000095367432" hidden="0" customWidth="1"/>
+    <x:col min="14" max="14" width="12.789999961853027" hidden="0" customWidth="1"/>
+    <x:col min="15" max="15" width="7.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="8.210000038146973" hidden="0" customWidth="1"/>
+    <x:col min="17" max="17" width="3.2300000190734863" hidden="0" customWidth="1"/>
+    <x:col min="18" max="18" width="7.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="19" max="19" width="19.25" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="7.400000095367432" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="21" customHeight="1">
@@ -1452,42 +1719,39 @@
         <x:v>year</x:v>
       </x:c>
       <x:c r="I1" s="4" t="str">
-        <x:v>advisor_email</x:v>
+        <x:v>course_name</x:v>
       </x:c>
       <x:c r="J1" s="4" t="str">
-        <x:v>course_name</x:v>
+        <x:v>difficulty_type</x:v>
       </x:c>
       <x:c r="K1" s="4" t="str">
-        <x:v>difficulty_type</x:v>
+        <x:v>difficulty_score</x:v>
       </x:c>
       <x:c r="L1" s="4" t="str">
-        <x:v>difficulty_score</x:v>
+        <x:v>attendance_status</x:v>
       </x:c>
       <x:c r="M1" s="4" t="str">
-        <x:v>attendance_status</x:v>
+        <x:v>preferred_support</x:v>
       </x:c>
       <x:c r="N1" s="4" t="str">
-        <x:v>preferred_support</x:v>
+        <x:v>follow_up_date</x:v>
       </x:c>
       <x:c r="O1" s="4" t="str">
-        <x:v>follow_up_date</x:v>
+        <x:v>risk_level</x:v>
       </x:c>
       <x:c r="P1" s="4" t="str">
-        <x:v>risk_level</x:v>
+        <x:v>risk_score</x:v>
       </x:c>
       <x:c r="Q1" s="4" t="str">
-        <x:v>risk_score</x:v>
+        <x:v>tags</x:v>
       </x:c>
       <x:c r="R1" s="4" t="str">
-        <x:v>tags</x:v>
+        <x:v>summary</x:v>
       </x:c>
       <x:c r="S1" s="4" t="str">
-        <x:v>summary</x:v>
+        <x:v>recommendations_json</x:v>
       </x:c>
       <x:c r="T1" s="4" t="str">
-        <x:v>recommendations_json</x:v>
-      </x:c>
-      <x:c r="U1" s="4" t="str">
         <x:v>raw_json</x:v>
       </x:c>
     </x:row>
@@ -1573,15 +1837,14 @@
     <x:col min="2" max="2" width="8.75" hidden="0" customWidth="1"/>
     <x:col min="3" max="3" width="8.75" hidden="0" customWidth="1"/>
     <x:col min="4" max="4" width="11.84000015258789" hidden="0" customWidth="1"/>
-    <x:col min="5" max="5" width="11.4399995803833" hidden="0" customWidth="1"/>
-    <x:col min="6" max="6" width="5.380000114440918" hidden="0" customWidth="1"/>
-    <x:col min="7" max="7" width="7" hidden="0" customWidth="1"/>
-    <x:col min="8" max="8" width="6.460000038146973" hidden="0" customWidth="1"/>
-    <x:col min="9" max="9" width="7.269999980926514" hidden="0" customWidth="1"/>
-    <x:col min="10" max="10" width="8.210000038146973" hidden="0" customWidth="1"/>
-    <x:col min="11" max="11" width="4.849999904632568" hidden="0" customWidth="1"/>
-    <x:col min="12" max="12" width="7.670000076293945" hidden="0" customWidth="1"/>
-    <x:col min="13" max="13" width="9.5600004196167" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="5.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="7" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="6.460000038146973" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="7.269999980926514" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="8.210000038146973" hidden="0" customWidth="1"/>
+    <x:col min="10" max="10" width="4.849999904632568" hidden="0" customWidth="1"/>
+    <x:col min="11" max="11" width="7.670000076293945" hidden="0" customWidth="1"/>
+    <x:col min="12" max="12" width="9.5600004196167" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="21" customHeight="1">
@@ -1598,30 +1861,27 @@
         <x:v>student_name</x:v>
       </x:c>
       <x:c r="E1" s="4" t="str">
-        <x:v>advisor_email</x:v>
+        <x:v>source</x:v>
       </x:c>
       <x:c r="F1" s="4" t="str">
-        <x:v>source</x:v>
+        <x:v>category</x:v>
       </x:c>
       <x:c r="G1" s="4" t="str">
-        <x:v>category</x:v>
+        <x:v>severity</x:v>
       </x:c>
       <x:c r="H1" s="4" t="str">
-        <x:v>severity</x:v>
+        <x:v>evidence</x:v>
       </x:c>
       <x:c r="I1" s="4" t="str">
-        <x:v>evidence</x:v>
+        <x:v>risk_score</x:v>
       </x:c>
       <x:c r="J1" s="4" t="str">
-        <x:v>risk_score</x:v>
+        <x:v>status</x:v>
       </x:c>
       <x:c r="K1" s="4" t="str">
-        <x:v>status</x:v>
+        <x:v>due_date</x:v>
       </x:c>
       <x:c r="L1" s="4" t="str">
-        <x:v>due_date</x:v>
-      </x:c>
-      <x:c r="M1" s="4" t="str">
         <x:v>resolved_at</x:v>
       </x:c>
     </x:row>

</xml_diff>